<commit_message>
Adding some data for Shallap and updates to param files
</commit_message>
<xml_diff>
--- a/Shallap/Parameters/VPAR_T.xlsx
+++ b/Shallap/Parameters/VPAR_T.xlsx
@@ -8,15 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\group\pelligrp\Project_folders\MountainWater\Tethys_Chloris\Workflow_dev\Scripts\Cat\TeC_Source_Code\Shallap\Parameters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D79E2B47-89AF-4060-9AEE-03EBEDC615C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3BCC811-A649-4238-A5AC-27AD474C5B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-5475" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -25,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Class</t>
   </si>
@@ -58,6 +67,12 @@
   </si>
   <si>
     <t>Cbare</t>
+  </si>
+  <si>
+    <t>Kbot</t>
+  </si>
+  <si>
+    <t>Krock</t>
   </si>
 </sst>
 </file>
@@ -406,7 +421,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.36328125" customWidth="1"/>
@@ -418,7 +433,7 @@
     <col min="7" max="7" width="6.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -440,8 +455,14 @@
       <c r="G1" t="s">
         <v>10</v>
       </c>
+      <c r="H1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -463,8 +484,14 @@
       <c r="G2">
         <v>0.2</v>
       </c>
+      <c r="H2">
+        <v>0.1</v>
+      </c>
+      <c r="I2">
+        <v>0.1</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -486,8 +513,14 @@
       <c r="G3">
         <v>0.3</v>
       </c>
+      <c r="H3">
+        <v>0.1</v>
+      </c>
+      <c r="I3">
+        <v>0.1</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -509,8 +542,14 @@
       <c r="G4">
         <v>0</v>
       </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -531,6 +570,12 @@
       </c>
       <c r="G5">
         <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0.1</v>
+      </c>
+      <c r="I5">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>